<commit_message>
UPDATE se agrega planilla con estaciones y se carga DF (aunque esta incorrecto)
</commit_message>
<xml_diff>
--- a/Outputs/RIO ASTABURUAGA EN CONO.xlsx
+++ b/Outputs/RIO ASTABURUAGA EN CONO.xlsx
@@ -76,13 +76,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,8 +110,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,7 +481,7 @@
       <c r="J2" t="n">
         <v>4130</v>
       </c>
-      <c r="K2"/>
+      <c r="K2" s="1"/>
       <c r="L2" t="n">
         <v>1979</v>
       </c>
@@ -520,7 +526,7 @@
       <c r="J3" t="n">
         <v>4130</v>
       </c>
-      <c r="K3"/>
+      <c r="K3" s="1"/>
       <c r="L3" t="n">
         <v>1980</v>
       </c>
@@ -565,7 +571,7 @@
       <c r="J4" t="n">
         <v>4130</v>
       </c>
-      <c r="K4"/>
+      <c r="K4" s="1"/>
       <c r="L4" t="n">
         <v>1980</v>
       </c>
@@ -610,7 +616,7 @@
       <c r="J5" t="n">
         <v>4130</v>
       </c>
-      <c r="K5"/>
+      <c r="K5" s="1"/>
       <c r="L5" t="n">
         <v>1980</v>
       </c>
@@ -655,7 +661,7 @@
       <c r="J6" t="n">
         <v>4130</v>
       </c>
-      <c r="K6"/>
+      <c r="K6" s="1"/>
       <c r="L6" t="n">
         <v>1980</v>
       </c>
@@ -700,7 +706,7 @@
       <c r="J7" t="n">
         <v>4130</v>
       </c>
-      <c r="K7"/>
+      <c r="K7" s="1"/>
       <c r="L7" t="n">
         <v>1981</v>
       </c>
@@ -745,7 +751,7 @@
       <c r="J8" t="n">
         <v>4130</v>
       </c>
-      <c r="K8"/>
+      <c r="K8" s="1"/>
       <c r="L8" t="n">
         <v>1981</v>
       </c>
@@ -790,7 +796,7 @@
       <c r="J9" t="n">
         <v>4130</v>
       </c>
-      <c r="K9"/>
+      <c r="K9" s="1"/>
       <c r="L9" t="n">
         <v>1981</v>
       </c>
@@ -835,7 +841,7 @@
       <c r="J10" t="n">
         <v>4130</v>
       </c>
-      <c r="K10"/>
+      <c r="K10" s="1"/>
       <c r="L10" t="n">
         <v>1981</v>
       </c>
@@ -880,7 +886,7 @@
       <c r="J11" t="n">
         <v>4130</v>
       </c>
-      <c r="K11"/>
+      <c r="K11" s="1"/>
       <c r="L11" t="n">
         <v>1981</v>
       </c>
@@ -925,7 +931,7 @@
       <c r="J12" t="n">
         <v>4130</v>
       </c>
-      <c r="K12"/>
+      <c r="K12" s="1"/>
       <c r="L12" t="n">
         <v>1982</v>
       </c>
@@ -970,7 +976,7 @@
       <c r="J13" t="n">
         <v>4130</v>
       </c>
-      <c r="K13"/>
+      <c r="K13" s="1"/>
       <c r="L13" t="n">
         <v>1982</v>
       </c>
@@ -1015,7 +1021,7 @@
       <c r="J14" t="n">
         <v>4130</v>
       </c>
-      <c r="K14"/>
+      <c r="K14" s="1"/>
       <c r="L14" t="n">
         <v>1982</v>
       </c>
@@ -1060,7 +1066,7 @@
       <c r="J15" t="n">
         <v>4130</v>
       </c>
-      <c r="K15"/>
+      <c r="K15" s="1"/>
       <c r="L15" t="n">
         <v>1982</v>
       </c>
@@ -1105,7 +1111,7 @@
       <c r="J16" t="n">
         <v>4130</v>
       </c>
-      <c r="K16"/>
+      <c r="K16" s="1"/>
       <c r="L16" t="n">
         <v>1982</v>
       </c>
@@ -1150,7 +1156,7 @@
       <c r="J17" t="n">
         <v>4130</v>
       </c>
-      <c r="K17"/>
+      <c r="K17" s="1"/>
       <c r="L17" t="n">
         <v>1982</v>
       </c>
@@ -1195,7 +1201,7 @@
       <c r="J18" t="n">
         <v>4130</v>
       </c>
-      <c r="K18"/>
+      <c r="K18" s="1"/>
       <c r="L18" t="n">
         <v>1982</v>
       </c>
@@ -1240,7 +1246,7 @@
       <c r="J19" t="n">
         <v>4130</v>
       </c>
-      <c r="K19"/>
+      <c r="K19" s="1"/>
       <c r="L19" t="n">
         <v>1983</v>
       </c>
@@ -1285,7 +1291,7 @@
       <c r="J20" t="n">
         <v>4130</v>
       </c>
-      <c r="K20"/>
+      <c r="K20" s="1"/>
       <c r="L20" t="n">
         <v>1983</v>
       </c>
@@ -1330,7 +1336,7 @@
       <c r="J21" t="n">
         <v>4130</v>
       </c>
-      <c r="K21"/>
+      <c r="K21" s="1"/>
       <c r="L21" t="n">
         <v>1983</v>
       </c>
@@ -1375,7 +1381,7 @@
       <c r="J22" t="n">
         <v>4130</v>
       </c>
-      <c r="K22"/>
+      <c r="K22" s="1"/>
       <c r="L22" t="n">
         <v>1983</v>
       </c>
@@ -1420,7 +1426,7 @@
       <c r="J23" t="n">
         <v>4130</v>
       </c>
-      <c r="K23"/>
+      <c r="K23" s="1"/>
       <c r="L23" t="n">
         <v>1983</v>
       </c>
@@ -1465,7 +1471,7 @@
       <c r="J24" t="n">
         <v>4130</v>
       </c>
-      <c r="K24"/>
+      <c r="K24" s="1"/>
       <c r="L24" t="n">
         <v>1983</v>
       </c>
@@ -1510,7 +1516,7 @@
       <c r="J25" t="n">
         <v>4130</v>
       </c>
-      <c r="K25"/>
+      <c r="K25" s="1"/>
       <c r="L25" t="n">
         <v>1983</v>
       </c>
@@ -1555,7 +1561,7 @@
       <c r="J26" t="n">
         <v>4130</v>
       </c>
-      <c r="K26"/>
+      <c r="K26" s="1"/>
       <c r="L26" t="n">
         <v>1984</v>
       </c>
@@ -1600,7 +1606,7 @@
       <c r="J27" t="n">
         <v>4130</v>
       </c>
-      <c r="K27"/>
+      <c r="K27" s="1"/>
       <c r="L27" t="n">
         <v>1984</v>
       </c>
@@ -1645,7 +1651,7 @@
       <c r="J28" t="n">
         <v>4130</v>
       </c>
-      <c r="K28"/>
+      <c r="K28" s="1"/>
       <c r="L28" t="n">
         <v>1984</v>
       </c>
@@ -1690,7 +1696,7 @@
       <c r="J29" t="n">
         <v>4130</v>
       </c>
-      <c r="K29"/>
+      <c r="K29" s="1"/>
       <c r="L29" t="n">
         <v>1984</v>
       </c>
@@ -1735,7 +1741,7 @@
       <c r="J30" t="n">
         <v>4130</v>
       </c>
-      <c r="K30"/>
+      <c r="K30" s="1"/>
       <c r="L30" t="n">
         <v>1984</v>
       </c>
@@ -1780,7 +1786,7 @@
       <c r="J31" t="n">
         <v>4130</v>
       </c>
-      <c r="K31"/>
+      <c r="K31" s="1"/>
       <c r="L31" t="n">
         <v>1984</v>
       </c>
@@ -1825,7 +1831,7 @@
       <c r="J32" t="n">
         <v>4130</v>
       </c>
-      <c r="K32"/>
+      <c r="K32" s="1"/>
       <c r="L32" t="n">
         <v>1985</v>
       </c>
@@ -1870,7 +1876,7 @@
       <c r="J33" t="n">
         <v>4130</v>
       </c>
-      <c r="K33"/>
+      <c r="K33" s="1"/>
       <c r="L33" t="n">
         <v>1985</v>
       </c>
@@ -1915,7 +1921,7 @@
       <c r="J34" t="n">
         <v>4130</v>
       </c>
-      <c r="K34"/>
+      <c r="K34" s="1"/>
       <c r="L34" t="n">
         <v>1985</v>
       </c>
@@ -1960,7 +1966,7 @@
       <c r="J35" t="n">
         <v>4130</v>
       </c>
-      <c r="K35"/>
+      <c r="K35" s="1"/>
       <c r="L35" t="n">
         <v>1985</v>
       </c>
@@ -2005,7 +2011,7 @@
       <c r="J36" t="n">
         <v>4130</v>
       </c>
-      <c r="K36"/>
+      <c r="K36" s="1"/>
       <c r="L36" t="n">
         <v>1985</v>
       </c>
@@ -2050,7 +2056,7 @@
       <c r="J37" t="n">
         <v>4130</v>
       </c>
-      <c r="K37"/>
+      <c r="K37" s="1"/>
       <c r="L37" t="n">
         <v>1985</v>
       </c>
@@ -2095,7 +2101,7 @@
       <c r="J38" t="n">
         <v>4130</v>
       </c>
-      <c r="K38"/>
+      <c r="K38" s="1"/>
       <c r="L38" t="n">
         <v>1986</v>
       </c>
@@ -2140,7 +2146,7 @@
       <c r="J39" t="n">
         <v>4130</v>
       </c>
-      <c r="K39"/>
+      <c r="K39" s="1"/>
       <c r="L39" t="n">
         <v>1986</v>
       </c>
@@ -2185,7 +2191,7 @@
       <c r="J40" t="n">
         <v>4130</v>
       </c>
-      <c r="K40"/>
+      <c r="K40" s="1"/>
       <c r="L40" t="n">
         <v>1986</v>
       </c>
@@ -2230,7 +2236,7 @@
       <c r="J41" t="n">
         <v>4130</v>
       </c>
-      <c r="K41"/>
+      <c r="K41" s="1"/>
       <c r="L41" t="n">
         <v>1986</v>
       </c>
@@ -2275,7 +2281,7 @@
       <c r="J42" t="n">
         <v>4130</v>
       </c>
-      <c r="K42"/>
+      <c r="K42" s="1"/>
       <c r="L42" t="n">
         <v>1986</v>
       </c>
@@ -2320,7 +2326,7 @@
       <c r="J43" t="n">
         <v>4130</v>
       </c>
-      <c r="K43"/>
+      <c r="K43" s="1"/>
       <c r="L43" t="n">
         <v>1986</v>
       </c>
@@ -2365,7 +2371,7 @@
       <c r="J44" t="n">
         <v>4130</v>
       </c>
-      <c r="K44"/>
+      <c r="K44" s="1"/>
       <c r="L44" t="n">
         <v>1986</v>
       </c>
@@ -2410,7 +2416,7 @@
       <c r="J45" t="n">
         <v>4130</v>
       </c>
-      <c r="K45"/>
+      <c r="K45" s="1"/>
       <c r="L45" t="n">
         <v>1986</v>
       </c>
@@ -2455,7 +2461,7 @@
       <c r="J46" t="n">
         <v>4130</v>
       </c>
-      <c r="K46"/>
+      <c r="K46" s="1"/>
       <c r="L46" t="n">
         <v>1987</v>
       </c>
@@ -2500,7 +2506,7 @@
       <c r="J47" t="n">
         <v>4130</v>
       </c>
-      <c r="K47"/>
+      <c r="K47" s="1"/>
       <c r="L47" t="n">
         <v>1987</v>
       </c>
@@ -2545,7 +2551,7 @@
       <c r="J48" t="n">
         <v>4130</v>
       </c>
-      <c r="K48"/>
+      <c r="K48" s="1"/>
       <c r="L48" t="n">
         <v>1987</v>
       </c>
@@ -2590,7 +2596,7 @@
       <c r="J49" t="n">
         <v>4130</v>
       </c>
-      <c r="K49"/>
+      <c r="K49" s="1"/>
       <c r="L49" t="n">
         <v>1987</v>
       </c>
@@ -2635,7 +2641,7 @@
       <c r="J50" t="n">
         <v>4130</v>
       </c>
-      <c r="K50"/>
+      <c r="K50" s="1"/>
       <c r="L50" t="n">
         <v>1987</v>
       </c>
@@ -2680,7 +2686,7 @@
       <c r="J51" t="n">
         <v>4130</v>
       </c>
-      <c r="K51"/>
+      <c r="K51" s="1"/>
       <c r="L51" t="n">
         <v>1988</v>
       </c>
@@ -2725,7 +2731,7 @@
       <c r="J52" t="n">
         <v>4130</v>
       </c>
-      <c r="K52"/>
+      <c r="K52" s="1"/>
       <c r="L52" t="n">
         <v>1988</v>
       </c>
@@ -2770,7 +2776,7 @@
       <c r="J53" t="n">
         <v>4130</v>
       </c>
-      <c r="K53"/>
+      <c r="K53" s="1"/>
       <c r="L53" t="n">
         <v>1988</v>
       </c>
@@ -2815,7 +2821,7 @@
       <c r="J54" t="n">
         <v>4130</v>
       </c>
-      <c r="K54"/>
+      <c r="K54" s="1"/>
       <c r="L54" t="n">
         <v>1988</v>
       </c>
@@ -2860,7 +2866,7 @@
       <c r="J55" t="n">
         <v>4130</v>
       </c>
-      <c r="K55"/>
+      <c r="K55" s="1"/>
       <c r="L55" t="n">
         <v>1988</v>
       </c>
@@ -2905,7 +2911,7 @@
       <c r="J56" t="n">
         <v>4130</v>
       </c>
-      <c r="K56"/>
+      <c r="K56" s="1"/>
       <c r="L56" t="n">
         <v>1989</v>
       </c>
@@ -2950,7 +2956,7 @@
       <c r="J57" t="n">
         <v>4130</v>
       </c>
-      <c r="K57"/>
+      <c r="K57" s="1"/>
       <c r="L57" t="n">
         <v>1989</v>
       </c>
@@ -2995,7 +3001,7 @@
       <c r="J58" t="n">
         <v>4130</v>
       </c>
-      <c r="K58"/>
+      <c r="K58" s="1"/>
       <c r="L58" t="n">
         <v>1989</v>
       </c>
@@ -3040,7 +3046,7 @@
       <c r="J59" t="n">
         <v>4130</v>
       </c>
-      <c r="K59"/>
+      <c r="K59" s="1"/>
       <c r="L59" t="n">
         <v>1989</v>
       </c>
@@ -3085,7 +3091,7 @@
       <c r="J60" t="n">
         <v>4130</v>
       </c>
-      <c r="K60"/>
+      <c r="K60" s="1"/>
       <c r="L60" t="n">
         <v>1989</v>
       </c>
@@ -3130,7 +3136,7 @@
       <c r="J61" t="n">
         <v>4130</v>
       </c>
-      <c r="K61"/>
+      <c r="K61" s="1"/>
       <c r="L61" t="n">
         <v>1989</v>
       </c>
@@ -3175,7 +3181,7 @@
       <c r="J62" t="n">
         <v>4130</v>
       </c>
-      <c r="K62"/>
+      <c r="K62" s="1"/>
       <c r="L62" t="n">
         <v>1990</v>
       </c>
@@ -3220,7 +3226,7 @@
       <c r="J63" t="n">
         <v>4130</v>
       </c>
-      <c r="K63"/>
+      <c r="K63" s="1"/>
       <c r="L63" t="n">
         <v>1990</v>
       </c>
@@ -3265,7 +3271,7 @@
       <c r="J64" t="n">
         <v>4130</v>
       </c>
-      <c r="K64"/>
+      <c r="K64" s="1"/>
       <c r="L64" t="n">
         <v>1990</v>
       </c>
@@ -3310,7 +3316,7 @@
       <c r="J65" t="n">
         <v>4130</v>
       </c>
-      <c r="K65"/>
+      <c r="K65" s="1"/>
       <c r="L65" t="n">
         <v>1990</v>
       </c>
@@ -3355,7 +3361,7 @@
       <c r="J66" t="n">
         <v>4130</v>
       </c>
-      <c r="K66"/>
+      <c r="K66" s="1"/>
       <c r="L66" t="n">
         <v>1990</v>
       </c>
@@ -3400,7 +3406,7 @@
       <c r="J67" t="n">
         <v>4130</v>
       </c>
-      <c r="K67"/>
+      <c r="K67" s="1"/>
       <c r="L67" t="n">
         <v>1990</v>
       </c>
@@ -3445,7 +3451,7 @@
       <c r="J68" t="n">
         <v>4130</v>
       </c>
-      <c r="K68"/>
+      <c r="K68" s="1"/>
       <c r="L68" t="n">
         <v>1991</v>
       </c>
@@ -3490,7 +3496,7 @@
       <c r="J69" t="n">
         <v>4130</v>
       </c>
-      <c r="K69"/>
+      <c r="K69" s="1"/>
       <c r="L69" t="n">
         <v>1991</v>
       </c>
@@ -3535,7 +3541,7 @@
       <c r="J70" t="n">
         <v>4130</v>
       </c>
-      <c r="K70"/>
+      <c r="K70" s="1"/>
       <c r="L70" t="n">
         <v>1991</v>
       </c>
@@ -3580,7 +3586,7 @@
       <c r="J71" t="n">
         <v>4130</v>
       </c>
-      <c r="K71"/>
+      <c r="K71" s="1"/>
       <c r="L71" t="n">
         <v>1991</v>
       </c>
@@ -3625,7 +3631,7 @@
       <c r="J72" t="n">
         <v>4130</v>
       </c>
-      <c r="K72"/>
+      <c r="K72" s="1"/>
       <c r="L72" t="n">
         <v>1991</v>
       </c>
@@ -3670,7 +3676,7 @@
       <c r="J73" t="n">
         <v>4130</v>
       </c>
-      <c r="K73"/>
+      <c r="K73" s="1"/>
       <c r="L73" t="n">
         <v>1991</v>
       </c>
@@ -3715,7 +3721,7 @@
       <c r="J74" t="n">
         <v>4130</v>
       </c>
-      <c r="K74"/>
+      <c r="K74" s="1"/>
       <c r="L74" t="n">
         <v>1991</v>
       </c>
@@ -3760,7 +3766,7 @@
       <c r="J75" t="n">
         <v>4130</v>
       </c>
-      <c r="K75"/>
+      <c r="K75" s="1"/>
       <c r="L75" t="n">
         <v>1991</v>
       </c>
@@ -3805,7 +3811,7 @@
       <c r="J76" t="n">
         <v>4130</v>
       </c>
-      <c r="K76"/>
+      <c r="K76" s="1"/>
       <c r="L76" t="n">
         <v>1991</v>
       </c>
@@ -3850,7 +3856,7 @@
       <c r="J77" t="n">
         <v>4130</v>
       </c>
-      <c r="K77"/>
+      <c r="K77" s="1"/>
       <c r="L77" t="n">
         <v>1992</v>
       </c>
@@ -3895,7 +3901,7 @@
       <c r="J78" t="n">
         <v>4130</v>
       </c>
-      <c r="K78"/>
+      <c r="K78" s="1"/>
       <c r="L78" t="n">
         <v>1992</v>
       </c>
@@ -3940,7 +3946,7 @@
       <c r="J79" t="n">
         <v>4130</v>
       </c>
-      <c r="K79"/>
+      <c r="K79" s="1"/>
       <c r="L79" t="n">
         <v>1992</v>
       </c>
@@ -3985,7 +3991,7 @@
       <c r="J80" t="n">
         <v>4130</v>
       </c>
-      <c r="K80"/>
+      <c r="K80" s="1"/>
       <c r="L80" t="n">
         <v>1992</v>
       </c>
@@ -4030,7 +4036,7 @@
       <c r="J81" t="n">
         <v>4130</v>
       </c>
-      <c r="K81"/>
+      <c r="K81" s="1"/>
       <c r="L81" t="n">
         <v>1993</v>
       </c>
@@ -4075,7 +4081,7 @@
       <c r="J82" t="n">
         <v>4130</v>
       </c>
-      <c r="K82"/>
+      <c r="K82" s="1"/>
       <c r="L82" t="n">
         <v>1993</v>
       </c>
@@ -4120,7 +4126,7 @@
       <c r="J83" t="n">
         <v>4130</v>
       </c>
-      <c r="K83"/>
+      <c r="K83" s="1"/>
       <c r="L83" t="n">
         <v>1993</v>
       </c>
@@ -4165,7 +4171,7 @@
       <c r="J84" t="n">
         <v>4130</v>
       </c>
-      <c r="K84"/>
+      <c r="K84" s="1"/>
       <c r="L84" t="n">
         <v>1993</v>
       </c>
@@ -4210,7 +4216,7 @@
       <c r="J85" t="n">
         <v>4130</v>
       </c>
-      <c r="K85"/>
+      <c r="K85" s="1"/>
       <c r="L85" t="n">
         <v>1993</v>
       </c>
@@ -4255,7 +4261,7 @@
       <c r="J86" t="n">
         <v>4130</v>
       </c>
-      <c r="K86"/>
+      <c r="K86" s="1"/>
       <c r="L86" t="n">
         <v>1993</v>
       </c>
@@ -4300,7 +4306,7 @@
       <c r="J87" t="n">
         <v>4130</v>
       </c>
-      <c r="K87"/>
+      <c r="K87" s="1"/>
       <c r="L87" t="n">
         <v>1993</v>
       </c>
@@ -4345,7 +4351,7 @@
       <c r="J88" t="n">
         <v>4130</v>
       </c>
-      <c r="K88"/>
+      <c r="K88" s="1"/>
       <c r="L88" t="n">
         <v>1993</v>
       </c>
@@ -4390,7 +4396,7 @@
       <c r="J89" t="n">
         <v>4130</v>
       </c>
-      <c r="K89"/>
+      <c r="K89" s="1"/>
       <c r="L89" t="n">
         <v>1993</v>
       </c>
@@ -4435,7 +4441,7 @@
       <c r="J90" t="n">
         <v>4130</v>
       </c>
-      <c r="K90"/>
+      <c r="K90" s="1"/>
       <c r="L90" t="n">
         <v>1994</v>
       </c>
@@ -4480,7 +4486,7 @@
       <c r="J91" t="n">
         <v>4130</v>
       </c>
-      <c r="K91"/>
+      <c r="K91" s="1"/>
       <c r="L91" t="n">
         <v>1994</v>
       </c>
@@ -4525,7 +4531,7 @@
       <c r="J92" t="n">
         <v>4130</v>
       </c>
-      <c r="K92"/>
+      <c r="K92" s="1"/>
       <c r="L92" t="n">
         <v>1994</v>
       </c>
@@ -4570,7 +4576,7 @@
       <c r="J93" t="n">
         <v>4130</v>
       </c>
-      <c r="K93"/>
+      <c r="K93" s="1"/>
       <c r="L93" t="n">
         <v>1994</v>
       </c>
@@ -4615,7 +4621,7 @@
       <c r="J94" t="n">
         <v>4130</v>
       </c>
-      <c r="K94"/>
+      <c r="K94" s="1"/>
       <c r="L94" t="n">
         <v>1994</v>
       </c>
@@ -4660,7 +4666,7 @@
       <c r="J95" t="n">
         <v>4130</v>
       </c>
-      <c r="K95"/>
+      <c r="K95" s="1"/>
       <c r="L95" t="n">
         <v>1994</v>
       </c>
@@ -4705,7 +4711,7 @@
       <c r="J96" t="n">
         <v>4130</v>
       </c>
-      <c r="K96"/>
+      <c r="K96" s="1"/>
       <c r="L96" t="n">
         <v>1994</v>
       </c>
@@ -4750,7 +4756,7 @@
       <c r="J97" t="n">
         <v>4130</v>
       </c>
-      <c r="K97"/>
+      <c r="K97" s="1"/>
       <c r="L97" t="n">
         <v>1994</v>
       </c>
@@ -4795,7 +4801,7 @@
       <c r="J98" t="n">
         <v>4130</v>
       </c>
-      <c r="K98"/>
+      <c r="K98" s="1"/>
       <c r="L98" t="n">
         <v>1994</v>
       </c>
@@ -4840,7 +4846,7 @@
       <c r="J99" t="n">
         <v>4130</v>
       </c>
-      <c r="K99"/>
+      <c r="K99" s="1"/>
       <c r="L99" t="n">
         <v>1994</v>
       </c>
@@ -4885,7 +4891,7 @@
       <c r="J100" t="n">
         <v>4130</v>
       </c>
-      <c r="K100"/>
+      <c r="K100" s="1"/>
       <c r="L100" t="n">
         <v>1994</v>
       </c>
@@ -4930,7 +4936,7 @@
       <c r="J101" t="n">
         <v>4130</v>
       </c>
-      <c r="K101"/>
+      <c r="K101" s="1"/>
       <c r="L101" t="n">
         <v>1995</v>
       </c>
@@ -4975,7 +4981,7 @@
       <c r="J102" t="n">
         <v>4130</v>
       </c>
-      <c r="K102"/>
+      <c r="K102" s="1"/>
       <c r="L102" t="n">
         <v>1995</v>
       </c>
@@ -5020,7 +5026,7 @@
       <c r="J103" t="n">
         <v>4130</v>
       </c>
-      <c r="K103"/>
+      <c r="K103" s="1"/>
       <c r="L103" t="n">
         <v>1995</v>
       </c>
@@ -5065,7 +5071,7 @@
       <c r="J104" t="n">
         <v>4130</v>
       </c>
-      <c r="K104"/>
+      <c r="K104" s="1"/>
       <c r="L104" t="n">
         <v>1995</v>
       </c>
@@ -5110,7 +5116,7 @@
       <c r="J105" t="n">
         <v>4130</v>
       </c>
-      <c r="K105"/>
+      <c r="K105" s="1"/>
       <c r="L105" t="n">
         <v>1995</v>
       </c>
@@ -5155,7 +5161,7 @@
       <c r="J106" t="n">
         <v>4130</v>
       </c>
-      <c r="K106"/>
+      <c r="K106" s="1"/>
       <c r="L106" t="n">
         <v>1995</v>
       </c>
@@ -5200,7 +5206,7 @@
       <c r="J107" t="n">
         <v>4130</v>
       </c>
-      <c r="K107"/>
+      <c r="K107" s="1"/>
       <c r="L107" t="n">
         <v>1995</v>
       </c>
@@ -5245,7 +5251,7 @@
       <c r="J108" t="n">
         <v>4130</v>
       </c>
-      <c r="K108"/>
+      <c r="K108" s="1"/>
       <c r="L108" t="n">
         <v>1995</v>
       </c>
@@ -5290,7 +5296,7 @@
       <c r="J109" t="n">
         <v>4130</v>
       </c>
-      <c r="K109"/>
+      <c r="K109" s="1"/>
       <c r="L109" t="n">
         <v>1995</v>
       </c>
@@ -5335,7 +5341,7 @@
       <c r="J110" t="n">
         <v>4130</v>
       </c>
-      <c r="K110"/>
+      <c r="K110" s="1"/>
       <c r="L110" t="n">
         <v>1996</v>
       </c>
@@ -5380,7 +5386,7 @@
       <c r="J111" t="n">
         <v>4130</v>
       </c>
-      <c r="K111"/>
+      <c r="K111" s="1"/>
       <c r="L111" t="n">
         <v>1996</v>
       </c>
@@ -5425,7 +5431,7 @@
       <c r="J112" t="n">
         <v>4130</v>
       </c>
-      <c r="K112"/>
+      <c r="K112" s="1"/>
       <c r="L112" t="n">
         <v>1996</v>
       </c>
@@ -5470,7 +5476,7 @@
       <c r="J113" t="n">
         <v>4130</v>
       </c>
-      <c r="K113"/>
+      <c r="K113" s="1"/>
       <c r="L113" t="n">
         <v>1996</v>
       </c>
@@ -5515,7 +5521,7 @@
       <c r="J114" t="n">
         <v>4130</v>
       </c>
-      <c r="K114"/>
+      <c r="K114" s="1"/>
       <c r="L114" t="n">
         <v>1996</v>
       </c>
@@ -5560,7 +5566,7 @@
       <c r="J115" t="n">
         <v>4130</v>
       </c>
-      <c r="K115"/>
+      <c r="K115" s="1"/>
       <c r="L115" t="n">
         <v>1997</v>
       </c>
@@ -5605,7 +5611,7 @@
       <c r="J116" t="n">
         <v>4130</v>
       </c>
-      <c r="K116"/>
+      <c r="K116" s="1"/>
       <c r="L116" t="n">
         <v>1997</v>
       </c>
@@ -5650,7 +5656,7 @@
       <c r="J117" t="n">
         <v>4130</v>
       </c>
-      <c r="K117"/>
+      <c r="K117" s="1"/>
       <c r="L117" t="n">
         <v>1997</v>
       </c>
@@ -5695,7 +5701,7 @@
       <c r="J118" t="n">
         <v>4130</v>
       </c>
-      <c r="K118"/>
+      <c r="K118" s="1"/>
       <c r="L118" t="n">
         <v>1997</v>
       </c>
@@ -5740,7 +5746,7 @@
       <c r="J119" t="n">
         <v>4130</v>
       </c>
-      <c r="K119"/>
+      <c r="K119" s="1"/>
       <c r="L119" t="n">
         <v>1997</v>
       </c>
@@ -5785,7 +5791,7 @@
       <c r="J120" t="n">
         <v>4130</v>
       </c>
-      <c r="K120"/>
+      <c r="K120" s="1"/>
       <c r="L120" t="n">
         <v>1998</v>
       </c>
@@ -5830,7 +5836,7 @@
       <c r="J121" t="n">
         <v>4130</v>
       </c>
-      <c r="K121"/>
+      <c r="K121" s="1"/>
       <c r="L121" t="n">
         <v>1998</v>
       </c>
@@ -5875,7 +5881,7 @@
       <c r="J122" t="n">
         <v>4130</v>
       </c>
-      <c r="K122"/>
+      <c r="K122" s="1"/>
       <c r="L122" t="n">
         <v>1998</v>
       </c>
@@ -5920,7 +5926,7 @@
       <c r="J123" t="n">
         <v>4130</v>
       </c>
-      <c r="K123"/>
+      <c r="K123" s="1"/>
       <c r="L123" t="n">
         <v>1998</v>
       </c>
@@ -5965,7 +5971,7 @@
       <c r="J124" t="n">
         <v>4130</v>
       </c>
-      <c r="K124"/>
+      <c r="K124" s="1"/>
       <c r="L124" t="n">
         <v>1998</v>
       </c>
@@ -6010,7 +6016,7 @@
       <c r="J125" t="n">
         <v>4130</v>
       </c>
-      <c r="K125"/>
+      <c r="K125" s="1"/>
       <c r="L125" t="n">
         <v>1999</v>
       </c>
@@ -6055,7 +6061,7 @@
       <c r="J126" t="n">
         <v>4130</v>
       </c>
-      <c r="K126"/>
+      <c r="K126" s="1"/>
       <c r="L126" t="n">
         <v>1999</v>
       </c>
@@ -6100,7 +6106,7 @@
       <c r="J127" t="n">
         <v>4130</v>
       </c>
-      <c r="K127"/>
+      <c r="K127" s="1"/>
       <c r="L127" t="n">
         <v>1999</v>
       </c>
@@ -6145,7 +6151,7 @@
       <c r="J128" t="n">
         <v>4130</v>
       </c>
-      <c r="K128"/>
+      <c r="K128" s="1"/>
       <c r="L128" t="n">
         <v>1999</v>
       </c>
@@ -6190,7 +6196,7 @@
       <c r="J129" t="n">
         <v>4130</v>
       </c>
-      <c r="K129"/>
+      <c r="K129" s="1"/>
       <c r="L129" t="n">
         <v>1999</v>
       </c>
@@ -6235,7 +6241,7 @@
       <c r="J130" t="n">
         <v>4130</v>
       </c>
-      <c r="K130"/>
+      <c r="K130" s="1"/>
       <c r="L130" t="n">
         <v>1999</v>
       </c>
@@ -6280,7 +6286,7 @@
       <c r="J131" t="n">
         <v>4130</v>
       </c>
-      <c r="K131"/>
+      <c r="K131" s="1"/>
       <c r="L131" t="n">
         <v>1999</v>
       </c>
@@ -6325,7 +6331,7 @@
       <c r="J132" t="n">
         <v>4130</v>
       </c>
-      <c r="K132"/>
+      <c r="K132" s="1"/>
       <c r="L132" t="n">
         <v>1999</v>
       </c>
@@ -6370,7 +6376,7 @@
       <c r="J133" t="n">
         <v>4130</v>
       </c>
-      <c r="K133"/>
+      <c r="K133" s="1"/>
       <c r="L133" t="n">
         <v>1999</v>
       </c>
@@ -6415,7 +6421,7 @@
       <c r="J134" t="n">
         <v>4130</v>
       </c>
-      <c r="K134"/>
+      <c r="K134" s="1"/>
       <c r="L134" t="n">
         <v>2000</v>
       </c>
@@ -6460,7 +6466,7 @@
       <c r="J135" t="n">
         <v>4130</v>
       </c>
-      <c r="K135"/>
+      <c r="K135" s="1"/>
       <c r="L135" t="n">
         <v>2000</v>
       </c>
@@ -6505,7 +6511,7 @@
       <c r="J136" t="n">
         <v>4130</v>
       </c>
-      <c r="K136"/>
+      <c r="K136" s="1"/>
       <c r="L136" t="n">
         <v>2000</v>
       </c>
@@ -6550,7 +6556,7 @@
       <c r="J137" t="n">
         <v>4130</v>
       </c>
-      <c r="K137"/>
+      <c r="K137" s="1"/>
       <c r="L137" t="n">
         <v>2000</v>
       </c>
@@ -6595,7 +6601,7 @@
       <c r="J138" t="n">
         <v>4130</v>
       </c>
-      <c r="K138"/>
+      <c r="K138" s="1"/>
       <c r="L138" t="n">
         <v>2000</v>
       </c>
@@ -6640,7 +6646,7 @@
       <c r="J139" t="n">
         <v>4130</v>
       </c>
-      <c r="K139"/>
+      <c r="K139" s="1"/>
       <c r="L139" t="n">
         <v>2000</v>
       </c>
@@ -6685,7 +6691,7 @@
       <c r="J140" t="n">
         <v>4130</v>
       </c>
-      <c r="K140"/>
+      <c r="K140" s="1"/>
       <c r="L140" t="n">
         <v>2000</v>
       </c>
@@ -6730,7 +6736,7 @@
       <c r="J141" t="n">
         <v>4130</v>
       </c>
-      <c r="K141"/>
+      <c r="K141" s="1"/>
       <c r="L141" t="n">
         <v>2000</v>
       </c>
@@ -6775,7 +6781,7 @@
       <c r="J142" t="n">
         <v>4130</v>
       </c>
-      <c r="K142"/>
+      <c r="K142" s="1"/>
       <c r="L142" t="n">
         <v>2001</v>
       </c>
@@ -6820,7 +6826,7 @@
       <c r="J143" t="n">
         <v>4130</v>
       </c>
-      <c r="K143"/>
+      <c r="K143" s="1"/>
       <c r="L143" t="n">
         <v>2001</v>
       </c>
@@ -6865,7 +6871,7 @@
       <c r="J144" t="n">
         <v>4130</v>
       </c>
-      <c r="K144"/>
+      <c r="K144" s="1"/>
       <c r="L144" t="n">
         <v>2001</v>
       </c>
@@ -6910,7 +6916,7 @@
       <c r="J145" t="n">
         <v>4130</v>
       </c>
-      <c r="K145"/>
+      <c r="K145" s="1"/>
       <c r="L145" t="n">
         <v>2001</v>
       </c>
@@ -6955,7 +6961,7 @@
       <c r="J146" t="n">
         <v>4130</v>
       </c>
-      <c r="K146"/>
+      <c r="K146" s="1"/>
       <c r="L146" t="n">
         <v>2001</v>
       </c>
@@ -7000,7 +7006,7 @@
       <c r="J147" t="n">
         <v>4130</v>
       </c>
-      <c r="K147"/>
+      <c r="K147" s="1"/>
       <c r="L147" t="n">
         <v>2001</v>
       </c>
@@ -7045,7 +7051,7 @@
       <c r="J148" t="n">
         <v>4130</v>
       </c>
-      <c r="K148"/>
+      <c r="K148" s="1"/>
       <c r="L148" t="n">
         <v>2001</v>
       </c>
@@ -7090,7 +7096,7 @@
       <c r="J149" t="n">
         <v>4130</v>
       </c>
-      <c r="K149"/>
+      <c r="K149" s="1"/>
       <c r="L149" t="n">
         <v>2001</v>
       </c>
@@ -7135,7 +7141,7 @@
       <c r="J150" t="n">
         <v>4130</v>
       </c>
-      <c r="K150"/>
+      <c r="K150" s="1"/>
       <c r="L150" t="n">
         <v>2001</v>
       </c>
@@ -7180,7 +7186,7 @@
       <c r="J151" t="n">
         <v>4130</v>
       </c>
-      <c r="K151"/>
+      <c r="K151" s="1"/>
       <c r="L151" t="n">
         <v>2002</v>
       </c>
@@ -7225,7 +7231,7 @@
       <c r="J152" t="n">
         <v>4130</v>
       </c>
-      <c r="K152"/>
+      <c r="K152" s="1"/>
       <c r="L152" t="n">
         <v>2002</v>
       </c>
@@ -7270,7 +7276,7 @@
       <c r="J153" t="n">
         <v>4130</v>
       </c>
-      <c r="K153"/>
+      <c r="K153" s="1"/>
       <c r="L153" t="n">
         <v>2002</v>
       </c>
@@ -7315,7 +7321,7 @@
       <c r="J154" t="n">
         <v>4130</v>
       </c>
-      <c r="K154"/>
+      <c r="K154" s="1"/>
       <c r="L154" t="n">
         <v>2002</v>
       </c>
@@ -7360,7 +7366,7 @@
       <c r="J155" t="n">
         <v>4130</v>
       </c>
-      <c r="K155"/>
+      <c r="K155" s="1"/>
       <c r="L155" t="n">
         <v>2003</v>
       </c>
@@ -7405,7 +7411,7 @@
       <c r="J156" t="n">
         <v>4130</v>
       </c>
-      <c r="K156"/>
+      <c r="K156" s="1"/>
       <c r="L156" t="n">
         <v>2003</v>
       </c>
@@ -7450,7 +7456,7 @@
       <c r="J157" t="n">
         <v>4130</v>
       </c>
-      <c r="K157"/>
+      <c r="K157" s="1"/>
       <c r="L157" t="n">
         <v>2003</v>
       </c>
@@ -7495,7 +7501,7 @@
       <c r="J158" t="n">
         <v>4130</v>
       </c>
-      <c r="K158"/>
+      <c r="K158" s="1"/>
       <c r="L158" t="n">
         <v>2003</v>
       </c>
@@ -7540,7 +7546,7 @@
       <c r="J159" t="n">
         <v>4130</v>
       </c>
-      <c r="K159"/>
+      <c r="K159" s="1"/>
       <c r="L159" t="n">
         <v>2003</v>
       </c>
@@ -7585,7 +7591,7 @@
       <c r="J160" t="n">
         <v>4130</v>
       </c>
-      <c r="K160"/>
+      <c r="K160" s="1"/>
       <c r="L160" t="n">
         <v>2003</v>
       </c>
@@ -7630,7 +7636,7 @@
       <c r="J161" t="n">
         <v>4130</v>
       </c>
-      <c r="K161"/>
+      <c r="K161" s="1"/>
       <c r="L161" t="n">
         <v>2003</v>
       </c>
@@ -7675,7 +7681,7 @@
       <c r="J162" t="n">
         <v>4130</v>
       </c>
-      <c r="K162"/>
+      <c r="K162" s="1"/>
       <c r="L162" t="n">
         <v>2004</v>
       </c>
@@ -7720,7 +7726,7 @@
       <c r="J163" t="n">
         <v>4130</v>
       </c>
-      <c r="K163"/>
+      <c r="K163" s="1"/>
       <c r="L163" t="n">
         <v>2004</v>
       </c>
@@ -7765,7 +7771,7 @@
       <c r="J164" t="n">
         <v>4130</v>
       </c>
-      <c r="K164"/>
+      <c r="K164" s="1"/>
       <c r="L164" t="n">
         <v>2004</v>
       </c>
@@ -7810,7 +7816,7 @@
       <c r="J165" t="n">
         <v>4130</v>
       </c>
-      <c r="K165"/>
+      <c r="K165" s="1"/>
       <c r="L165" t="n">
         <v>2004</v>
       </c>
@@ -7855,7 +7861,7 @@
       <c r="J166" t="n">
         <v>4130</v>
       </c>
-      <c r="K166"/>
+      <c r="K166" s="1"/>
       <c r="L166" t="n">
         <v>2004</v>
       </c>
@@ -7900,7 +7906,7 @@
       <c r="J167" t="n">
         <v>4130</v>
       </c>
-      <c r="K167"/>
+      <c r="K167" s="1"/>
       <c r="L167" t="n">
         <v>2005</v>
       </c>
@@ -7945,7 +7951,7 @@
       <c r="J168" t="n">
         <v>4130</v>
       </c>
-      <c r="K168"/>
+      <c r="K168" s="1"/>
       <c r="L168" t="n">
         <v>2005</v>
       </c>
@@ -7990,7 +7996,7 @@
       <c r="J169" t="n">
         <v>4130</v>
       </c>
-      <c r="K169"/>
+      <c r="K169" s="1"/>
       <c r="L169" t="n">
         <v>2005</v>
       </c>
@@ -8035,7 +8041,7 @@
       <c r="J170" t="n">
         <v>4130</v>
       </c>
-      <c r="K170"/>
+      <c r="K170" s="1"/>
       <c r="L170" t="n">
         <v>2005</v>
       </c>
@@ -8080,7 +8086,7 @@
       <c r="J171" t="n">
         <v>4130</v>
       </c>
-      <c r="K171"/>
+      <c r="K171" s="1"/>
       <c r="L171" t="n">
         <v>2006</v>
       </c>
@@ -8125,7 +8131,7 @@
       <c r="J172" t="n">
         <v>4130</v>
       </c>
-      <c r="K172"/>
+      <c r="K172" s="1"/>
       <c r="L172" t="n">
         <v>2006</v>
       </c>
@@ -8170,7 +8176,7 @@
       <c r="J173" t="n">
         <v>4130</v>
       </c>
-      <c r="K173"/>
+      <c r="K173" s="1"/>
       <c r="L173" t="n">
         <v>2006</v>
       </c>
@@ -8215,7 +8221,7 @@
       <c r="J174" t="n">
         <v>4130</v>
       </c>
-      <c r="K174"/>
+      <c r="K174" s="1"/>
       <c r="L174" t="n">
         <v>2006</v>
       </c>
@@ -8260,7 +8266,7 @@
       <c r="J175" t="n">
         <v>4130</v>
       </c>
-      <c r="K175"/>
+      <c r="K175" s="1"/>
       <c r="L175" t="n">
         <v>2006</v>
       </c>
@@ -8305,7 +8311,7 @@
       <c r="J176" t="n">
         <v>4130</v>
       </c>
-      <c r="K176"/>
+      <c r="K176" s="1"/>
       <c r="L176" t="n">
         <v>2006</v>
       </c>
@@ -8350,7 +8356,7 @@
       <c r="J177" t="n">
         <v>4130</v>
       </c>
-      <c r="K177"/>
+      <c r="K177" s="1"/>
       <c r="L177" t="n">
         <v>2006</v>
       </c>
@@ -8395,7 +8401,7 @@
       <c r="J178" t="n">
         <v>4130</v>
       </c>
-      <c r="K178"/>
+      <c r="K178" s="1"/>
       <c r="L178" t="n">
         <v>2006</v>
       </c>
@@ -8440,7 +8446,7 @@
       <c r="J179" t="n">
         <v>4130</v>
       </c>
-      <c r="K179"/>
+      <c r="K179" s="1"/>
       <c r="L179" t="n">
         <v>2006</v>
       </c>
@@ -8485,7 +8491,7 @@
       <c r="J180" t="n">
         <v>4130</v>
       </c>
-      <c r="K180"/>
+      <c r="K180" s="1"/>
       <c r="L180" t="n">
         <v>2008</v>
       </c>
@@ -8530,7 +8536,7 @@
       <c r="J181" t="n">
         <v>4130</v>
       </c>
-      <c r="K181"/>
+      <c r="K181" s="1"/>
       <c r="L181" t="n">
         <v>2009</v>
       </c>
@@ -8575,7 +8581,7 @@
       <c r="J182" t="n">
         <v>4130</v>
       </c>
-      <c r="K182"/>
+      <c r="K182" s="1"/>
       <c r="L182" t="n">
         <v>2009</v>
       </c>
@@ -8620,7 +8626,7 @@
       <c r="J183" t="n">
         <v>4130</v>
       </c>
-      <c r="K183"/>
+      <c r="K183" s="1"/>
       <c r="L183" t="n">
         <v>2009</v>
       </c>
@@ -8665,7 +8671,7 @@
       <c r="J184" t="n">
         <v>4130</v>
       </c>
-      <c r="K184"/>
+      <c r="K184" s="1"/>
       <c r="L184" t="n">
         <v>2009</v>
       </c>
@@ -8710,7 +8716,7 @@
       <c r="J185" t="n">
         <v>4130</v>
       </c>
-      <c r="K185"/>
+      <c r="K185" s="1"/>
       <c r="L185" t="n">
         <v>2009</v>
       </c>
@@ -8755,7 +8761,7 @@
       <c r="J186" t="n">
         <v>4130</v>
       </c>
-      <c r="K186"/>
+      <c r="K186" s="1"/>
       <c r="L186" t="n">
         <v>2009</v>
       </c>
@@ -8800,7 +8806,7 @@
       <c r="J187" t="n">
         <v>4130</v>
       </c>
-      <c r="K187"/>
+      <c r="K187" s="1"/>
       <c r="L187" t="n">
         <v>2009</v>
       </c>
@@ -8845,7 +8851,7 @@
       <c r="J188" t="n">
         <v>4130</v>
       </c>
-      <c r="K188"/>
+      <c r="K188" s="1"/>
       <c r="L188" t="n">
         <v>2010</v>
       </c>
@@ -8890,7 +8896,7 @@
       <c r="J189" t="n">
         <v>4130</v>
       </c>
-      <c r="K189"/>
+      <c r="K189" s="1"/>
       <c r="L189" t="n">
         <v>2010</v>
       </c>
@@ -8935,7 +8941,7 @@
       <c r="J190" t="n">
         <v>4130</v>
       </c>
-      <c r="K190"/>
+      <c r="K190" s="1"/>
       <c r="L190" t="n">
         <v>2010</v>
       </c>
@@ -8980,7 +8986,7 @@
       <c r="J191" t="n">
         <v>4130</v>
       </c>
-      <c r="K191"/>
+      <c r="K191" s="1"/>
       <c r="L191" t="n">
         <v>2010</v>
       </c>
@@ -9025,7 +9031,7 @@
       <c r="J192" t="n">
         <v>4130</v>
       </c>
-      <c r="K192"/>
+      <c r="K192" s="1"/>
       <c r="L192" t="n">
         <v>2010</v>
       </c>
@@ -9070,7 +9076,7 @@
       <c r="J193" t="n">
         <v>4130</v>
       </c>
-      <c r="K193"/>
+      <c r="K193" s="1"/>
       <c r="L193" t="n">
         <v>2010</v>
       </c>
@@ -9115,7 +9121,7 @@
       <c r="J194" t="n">
         <v>4130</v>
       </c>
-      <c r="K194"/>
+      <c r="K194" s="1"/>
       <c r="L194" t="n">
         <v>2010</v>
       </c>
@@ -9160,7 +9166,7 @@
       <c r="J195" t="n">
         <v>4130</v>
       </c>
-      <c r="K195"/>
+      <c r="K195" s="1"/>
       <c r="L195" t="n">
         <v>2010</v>
       </c>
@@ -9205,7 +9211,7 @@
       <c r="J196" t="n">
         <v>4130</v>
       </c>
-      <c r="K196"/>
+      <c r="K196" s="1"/>
       <c r="L196" t="n">
         <v>2010</v>
       </c>
@@ -9250,7 +9256,7 @@
       <c r="J197" t="n">
         <v>4130</v>
       </c>
-      <c r="K197"/>
+      <c r="K197" s="1"/>
       <c r="L197" t="n">
         <v>2011</v>
       </c>
@@ -9295,7 +9301,7 @@
       <c r="J198" t="n">
         <v>4130</v>
       </c>
-      <c r="K198"/>
+      <c r="K198" s="1"/>
       <c r="L198" t="n">
         <v>2011</v>
       </c>
@@ -9340,7 +9346,7 @@
       <c r="J199" t="n">
         <v>4130</v>
       </c>
-      <c r="K199"/>
+      <c r="K199" s="1"/>
       <c r="L199" t="n">
         <v>2011</v>
       </c>
@@ -9385,7 +9391,7 @@
       <c r="J200" t="n">
         <v>4130</v>
       </c>
-      <c r="K200"/>
+      <c r="K200" s="1"/>
       <c r="L200" t="n">
         <v>2011</v>
       </c>
@@ -9430,7 +9436,7 @@
       <c r="J201" t="n">
         <v>4130</v>
       </c>
-      <c r="K201"/>
+      <c r="K201" s="1"/>
       <c r="L201" t="n">
         <v>2011</v>
       </c>
@@ -9475,7 +9481,7 @@
       <c r="J202" t="n">
         <v>4130</v>
       </c>
-      <c r="K202"/>
+      <c r="K202" s="1"/>
       <c r="L202" t="n">
         <v>2011</v>
       </c>
@@ -9520,7 +9526,7 @@
       <c r="J203" t="n">
         <v>4130</v>
       </c>
-      <c r="K203"/>
+      <c r="K203" s="1"/>
       <c r="L203" t="n">
         <v>2011</v>
       </c>
@@ -9565,7 +9571,7 @@
       <c r="J204" t="n">
         <v>4130</v>
       </c>
-      <c r="K204"/>
+      <c r="K204" s="1"/>
       <c r="L204" t="n">
         <v>2011</v>
       </c>
@@ -9610,7 +9616,7 @@
       <c r="J205" t="n">
         <v>4130</v>
       </c>
-      <c r="K205"/>
+      <c r="K205" s="1"/>
       <c r="L205" t="n">
         <v>2012</v>
       </c>
@@ -9655,7 +9661,7 @@
       <c r="J206" t="n">
         <v>4130</v>
       </c>
-      <c r="K206"/>
+      <c r="K206" s="1"/>
       <c r="L206" t="n">
         <v>2012</v>
       </c>
@@ -9700,7 +9706,7 @@
       <c r="J207" t="n">
         <v>4130</v>
       </c>
-      <c r="K207"/>
+      <c r="K207" s="1"/>
       <c r="L207" t="n">
         <v>2012</v>
       </c>
@@ -9745,7 +9751,7 @@
       <c r="J208" t="n">
         <v>4130</v>
       </c>
-      <c r="K208"/>
+      <c r="K208" s="1"/>
       <c r="L208" t="n">
         <v>2012</v>
       </c>
@@ -9790,7 +9796,7 @@
       <c r="J209" t="n">
         <v>4130</v>
       </c>
-      <c r="K209"/>
+      <c r="K209" s="1"/>
       <c r="L209" t="n">
         <v>2012</v>
       </c>
@@ -9835,7 +9841,7 @@
       <c r="J210" t="n">
         <v>4130</v>
       </c>
-      <c r="K210"/>
+      <c r="K210" s="1"/>
       <c r="L210" t="n">
         <v>2012</v>
       </c>
@@ -9880,7 +9886,7 @@
       <c r="J211" t="n">
         <v>4130</v>
       </c>
-      <c r="K211"/>
+      <c r="K211" s="1"/>
       <c r="L211" t="n">
         <v>2012</v>
       </c>
@@ -9925,7 +9931,7 @@
       <c r="J212" t="n">
         <v>4130</v>
       </c>
-      <c r="K212"/>
+      <c r="K212" s="1"/>
       <c r="L212" t="n">
         <v>2012</v>
       </c>
@@ -9970,7 +9976,7 @@
       <c r="J213" t="n">
         <v>4130</v>
       </c>
-      <c r="K213"/>
+      <c r="K213" s="1"/>
       <c r="L213" t="n">
         <v>2012</v>
       </c>
@@ -10015,7 +10021,7 @@
       <c r="J214" t="n">
         <v>4130</v>
       </c>
-      <c r="K214"/>
+      <c r="K214" s="1"/>
       <c r="L214" t="n">
         <v>2012</v>
       </c>
@@ -10060,7 +10066,7 @@
       <c r="J215" t="n">
         <v>4130</v>
       </c>
-      <c r="K215"/>
+      <c r="K215" s="1"/>
       <c r="L215" t="n">
         <v>2012</v>
       </c>
@@ -10105,7 +10111,7 @@
       <c r="J216" t="n">
         <v>4130</v>
       </c>
-      <c r="K216"/>
+      <c r="K216" s="1"/>
       <c r="L216" t="n">
         <v>2013</v>
       </c>
@@ -10150,7 +10156,7 @@
       <c r="J217" t="n">
         <v>4130</v>
       </c>
-      <c r="K217"/>
+      <c r="K217" s="1"/>
       <c r="L217" t="n">
         <v>2013</v>
       </c>
@@ -10195,7 +10201,7 @@
       <c r="J218" t="n">
         <v>4130</v>
       </c>
-      <c r="K218"/>
+      <c r="K218" s="1"/>
       <c r="L218" t="n">
         <v>2013</v>
       </c>
@@ -10240,7 +10246,7 @@
       <c r="J219" t="n">
         <v>4130</v>
       </c>
-      <c r="K219"/>
+      <c r="K219" s="1"/>
       <c r="L219" t="n">
         <v>2013</v>
       </c>
@@ -10285,7 +10291,7 @@
       <c r="J220" t="n">
         <v>4130</v>
       </c>
-      <c r="K220"/>
+      <c r="K220" s="1"/>
       <c r="L220" t="n">
         <v>2013</v>
       </c>
@@ -10330,7 +10336,7 @@
       <c r="J221" t="n">
         <v>4130</v>
       </c>
-      <c r="K221"/>
+      <c r="K221" s="1"/>
       <c r="L221" t="n">
         <v>2013</v>
       </c>
@@ -10375,7 +10381,7 @@
       <c r="J222" t="n">
         <v>4130</v>
       </c>
-      <c r="K222"/>
+      <c r="K222" s="1"/>
       <c r="L222" t="n">
         <v>2013</v>
       </c>
@@ -10420,7 +10426,7 @@
       <c r="J223" t="n">
         <v>4130</v>
       </c>
-      <c r="K223"/>
+      <c r="K223" s="1"/>
       <c r="L223" t="n">
         <v>2013</v>
       </c>
@@ -10465,7 +10471,7 @@
       <c r="J224" t="n">
         <v>4130</v>
       </c>
-      <c r="K224"/>
+      <c r="K224" s="1"/>
       <c r="L224" t="n">
         <v>2013</v>
       </c>
@@ -10510,7 +10516,7 @@
       <c r="J225" t="n">
         <v>4130</v>
       </c>
-      <c r="K225"/>
+      <c r="K225" s="1"/>
       <c r="L225" t="n">
         <v>2013</v>
       </c>
@@ -10555,7 +10561,7 @@
       <c r="J226" t="n">
         <v>4130</v>
       </c>
-      <c r="K226"/>
+      <c r="K226" s="1"/>
       <c r="L226" t="n">
         <v>2014</v>
       </c>
@@ -10600,7 +10606,7 @@
       <c r="J227" t="n">
         <v>4130</v>
       </c>
-      <c r="K227"/>
+      <c r="K227" s="1"/>
       <c r="L227" t="n">
         <v>2014</v>
       </c>
@@ -10645,7 +10651,7 @@
       <c r="J228" t="n">
         <v>4130</v>
       </c>
-      <c r="K228"/>
+      <c r="K228" s="1"/>
       <c r="L228" t="n">
         <v>2014</v>
       </c>
@@ -10690,7 +10696,7 @@
       <c r="J229" t="n">
         <v>4130</v>
       </c>
-      <c r="K229"/>
+      <c r="K229" s="1"/>
       <c r="L229" t="n">
         <v>2014</v>
       </c>
@@ -10735,7 +10741,7 @@
       <c r="J230" t="n">
         <v>4130</v>
       </c>
-      <c r="K230"/>
+      <c r="K230" s="1"/>
       <c r="L230" t="n">
         <v>2014</v>
       </c>
@@ -10780,7 +10786,7 @@
       <c r="J231" t="n">
         <v>4130</v>
       </c>
-      <c r="K231"/>
+      <c r="K231" s="1"/>
       <c r="L231" t="n">
         <v>2014</v>
       </c>
@@ -10825,7 +10831,7 @@
       <c r="J232" t="n">
         <v>4130</v>
       </c>
-      <c r="K232"/>
+      <c r="K232" s="1"/>
       <c r="L232" t="n">
         <v>2014</v>
       </c>
@@ -10870,7 +10876,7 @@
       <c r="J233" t="n">
         <v>4130</v>
       </c>
-      <c r="K233"/>
+      <c r="K233" s="1"/>
       <c r="L233" t="n">
         <v>2015</v>
       </c>
@@ -10915,7 +10921,7 @@
       <c r="J234" t="n">
         <v>4130</v>
       </c>
-      <c r="K234"/>
+      <c r="K234" s="1"/>
       <c r="L234" t="n">
         <v>2015</v>
       </c>
@@ -10960,7 +10966,7 @@
       <c r="J235" t="n">
         <v>4130</v>
       </c>
-      <c r="K235"/>
+      <c r="K235" s="1"/>
       <c r="L235" t="n">
         <v>2015</v>
       </c>
@@ -11005,7 +11011,7 @@
       <c r="J236" t="n">
         <v>4130</v>
       </c>
-      <c r="K236"/>
+      <c r="K236" s="1"/>
       <c r="L236" t="n">
         <v>2015</v>
       </c>
@@ -11050,7 +11056,7 @@
       <c r="J237" t="n">
         <v>4130</v>
       </c>
-      <c r="K237"/>
+      <c r="K237" s="1"/>
       <c r="L237" t="n">
         <v>2015</v>
       </c>
@@ -11095,7 +11101,7 @@
       <c r="J238" t="n">
         <v>4130</v>
       </c>
-      <c r="K238"/>
+      <c r="K238" s="1"/>
       <c r="L238" t="n">
         <v>2016</v>
       </c>
@@ -11140,7 +11146,7 @@
       <c r="J239" t="n">
         <v>4130</v>
       </c>
-      <c r="K239"/>
+      <c r="K239" s="1"/>
       <c r="L239" t="n">
         <v>2016</v>
       </c>
@@ -11185,7 +11191,7 @@
       <c r="J240" t="n">
         <v>4130</v>
       </c>
-      <c r="K240"/>
+      <c r="K240" s="1"/>
       <c r="L240" t="n">
         <v>2016</v>
       </c>
@@ -11230,7 +11236,7 @@
       <c r="J241" t="n">
         <v>4130</v>
       </c>
-      <c r="K241"/>
+      <c r="K241" s="1"/>
       <c r="L241" t="n">
         <v>2016</v>
       </c>
@@ -11275,7 +11281,7 @@
       <c r="J242" t="n">
         <v>4130</v>
       </c>
-      <c r="K242"/>
+      <c r="K242" s="1"/>
       <c r="L242" t="n">
         <v>2016</v>
       </c>
@@ -11320,7 +11326,7 @@
       <c r="J243" t="n">
         <v>4130</v>
       </c>
-      <c r="K243"/>
+      <c r="K243" s="1"/>
       <c r="L243" t="n">
         <v>2016</v>
       </c>
@@ -11365,7 +11371,7 @@
       <c r="J244" t="n">
         <v>4130</v>
       </c>
-      <c r="K244"/>
+      <c r="K244" s="1"/>
       <c r="L244" t="n">
         <v>2017</v>
       </c>
@@ -11410,7 +11416,7 @@
       <c r="J245" t="n">
         <v>4130</v>
       </c>
-      <c r="K245"/>
+      <c r="K245" s="1"/>
       <c r="L245" t="n">
         <v>2017</v>
       </c>
@@ -11455,7 +11461,7 @@
       <c r="J246" t="n">
         <v>4130</v>
       </c>
-      <c r="K246"/>
+      <c r="K246" s="1"/>
       <c r="L246" t="n">
         <v>2017</v>
       </c>
@@ -11500,7 +11506,7 @@
       <c r="J247" t="n">
         <v>4130</v>
       </c>
-      <c r="K247"/>
+      <c r="K247" s="1"/>
       <c r="L247" t="n">
         <v>2017</v>
       </c>
@@ -11545,7 +11551,7 @@
       <c r="J248" t="n">
         <v>4130</v>
       </c>
-      <c r="K248"/>
+      <c r="K248" s="1"/>
       <c r="L248" t="n">
         <v>2018</v>
       </c>
@@ -11590,7 +11596,7 @@
       <c r="J249" t="n">
         <v>4130</v>
       </c>
-      <c r="K249"/>
+      <c r="K249" s="1"/>
       <c r="L249" t="n">
         <v>2018</v>
       </c>
@@ -11635,7 +11641,7 @@
       <c r="J250" t="n">
         <v>4130</v>
       </c>
-      <c r="K250"/>
+      <c r="K250" s="1"/>
       <c r="L250" t="n">
         <v>2019</v>
       </c>
@@ -11680,7 +11686,7 @@
       <c r="J251" t="n">
         <v>4130</v>
       </c>
-      <c r="K251"/>
+      <c r="K251" s="1"/>
       <c r="L251" t="n">
         <v>2019</v>
       </c>
@@ -11725,7 +11731,7 @@
       <c r="J252" t="n">
         <v>4130</v>
       </c>
-      <c r="K252"/>
+      <c r="K252" s="1"/>
       <c r="L252" t="n">
         <v>2019</v>
       </c>
@@ -11770,7 +11776,7 @@
       <c r="J253" t="n">
         <v>4130</v>
       </c>
-      <c r="K253"/>
+      <c r="K253" s="1"/>
       <c r="L253" t="n">
         <v>2019</v>
       </c>
@@ -11815,7 +11821,7 @@
       <c r="J254" t="n">
         <v>4130</v>
       </c>
-      <c r="K254"/>
+      <c r="K254" s="1"/>
       <c r="L254" t="n">
         <v>2019</v>
       </c>
@@ -11860,7 +11866,7 @@
       <c r="J255" t="n">
         <v>4130</v>
       </c>
-      <c r="K255"/>
+      <c r="K255" s="1"/>
       <c r="L255" t="n">
         <v>2019</v>
       </c>
@@ -11905,7 +11911,7 @@
       <c r="J256" t="n">
         <v>4130</v>
       </c>
-      <c r="K256"/>
+      <c r="K256" s="1"/>
       <c r="L256" t="n">
         <v>2019</v>
       </c>
@@ -11950,7 +11956,7 @@
       <c r="J257" t="n">
         <v>4130</v>
       </c>
-      <c r="K257"/>
+      <c r="K257" s="1"/>
       <c r="L257" t="n">
         <v>2019</v>
       </c>
@@ -11995,7 +12001,7 @@
       <c r="J258" t="n">
         <v>4130</v>
       </c>
-      <c r="K258"/>
+      <c r="K258" s="1"/>
       <c r="L258" t="n">
         <v>2019</v>
       </c>
@@ -12040,7 +12046,7 @@
       <c r="J259" t="n">
         <v>4130</v>
       </c>
-      <c r="K259"/>
+      <c r="K259" s="1"/>
       <c r="L259" t="n">
         <v>2020</v>
       </c>
@@ -12085,7 +12091,7 @@
       <c r="J260" t="n">
         <v>4130</v>
       </c>
-      <c r="K260"/>
+      <c r="K260" s="1"/>
       <c r="L260" t="n">
         <v>2020</v>
       </c>
@@ -12130,7 +12136,7 @@
       <c r="J261" t="n">
         <v>4130</v>
       </c>
-      <c r="K261"/>
+      <c r="K261" s="1"/>
       <c r="L261" t="n">
         <v>2020</v>
       </c>
@@ -12175,7 +12181,7 @@
       <c r="J262" t="n">
         <v>4130</v>
       </c>
-      <c r="K262"/>
+      <c r="K262" s="1"/>
       <c r="L262" t="n">
         <v>2020</v>
       </c>
@@ -12220,7 +12226,7 @@
       <c r="J263" t="n">
         <v>4130</v>
       </c>
-      <c r="K263"/>
+      <c r="K263" s="1"/>
       <c r="L263" t="n">
         <v>2020</v>
       </c>
@@ -12265,7 +12271,7 @@
       <c r="J264" t="n">
         <v>4130</v>
       </c>
-      <c r="K264"/>
+      <c r="K264" s="1"/>
       <c r="L264" t="n">
         <v>2020</v>
       </c>
@@ -12310,7 +12316,7 @@
       <c r="J265" t="n">
         <v>4130</v>
       </c>
-      <c r="K265"/>
+      <c r="K265" s="1"/>
       <c r="L265" t="n">
         <v>2020</v>
       </c>
@@ -12355,7 +12361,7 @@
       <c r="J266" t="n">
         <v>4130</v>
       </c>
-      <c r="K266"/>
+      <c r="K266" s="1"/>
       <c r="L266" t="n">
         <v>2020</v>
       </c>
@@ -12400,7 +12406,7 @@
       <c r="J267" t="n">
         <v>4130</v>
       </c>
-      <c r="K267"/>
+      <c r="K267" s="1"/>
       <c r="L267" t="n">
         <v>2020</v>
       </c>
@@ -12445,7 +12451,7 @@
       <c r="J268" t="n">
         <v>4130</v>
       </c>
-      <c r="K268"/>
+      <c r="K268" s="1"/>
       <c r="L268" t="n">
         <v>2020</v>
       </c>
@@ -12490,7 +12496,7 @@
       <c r="J269" t="n">
         <v>4130</v>
       </c>
-      <c r="K269"/>
+      <c r="K269" s="1"/>
       <c r="L269" t="n">
         <v>2021</v>
       </c>
@@ -12535,7 +12541,7 @@
       <c r="J270" t="n">
         <v>4130</v>
       </c>
-      <c r="K270"/>
+      <c r="K270" s="1"/>
       <c r="L270" t="n">
         <v>2021</v>
       </c>
@@ -12580,7 +12586,7 @@
       <c r="J271" t="n">
         <v>4130</v>
       </c>
-      <c r="K271"/>
+      <c r="K271" s="1"/>
       <c r="L271" t="n">
         <v>2021</v>
       </c>
@@ -12625,7 +12631,7 @@
       <c r="J272" t="n">
         <v>4130</v>
       </c>
-      <c r="K272"/>
+      <c r="K272" s="1"/>
       <c r="L272" t="n">
         <v>2021</v>
       </c>
@@ -12670,7 +12676,7 @@
       <c r="J273" t="n">
         <v>4130</v>
       </c>
-      <c r="K273"/>
+      <c r="K273" s="1"/>
       <c r="L273" t="n">
         <v>2021</v>
       </c>
@@ -12715,7 +12721,7 @@
       <c r="J274" t="n">
         <v>4130</v>
       </c>
-      <c r="K274"/>
+      <c r="K274" s="1"/>
       <c r="L274" t="n">
         <v>2021</v>
       </c>
@@ -12760,7 +12766,7 @@
       <c r="J275" t="n">
         <v>4130</v>
       </c>
-      <c r="K275"/>
+      <c r="K275" s="1"/>
       <c r="L275" t="n">
         <v>2021</v>
       </c>
@@ -12805,7 +12811,7 @@
       <c r="J276" t="n">
         <v>4130</v>
       </c>
-      <c r="K276"/>
+      <c r="K276" s="1"/>
       <c r="L276" t="n">
         <v>2021</v>
       </c>
@@ -12850,7 +12856,7 @@
       <c r="J277" t="n">
         <v>4130</v>
       </c>
-      <c r="K277"/>
+      <c r="K277" s="1"/>
       <c r="L277" t="n">
         <v>2022</v>
       </c>
@@ -12895,7 +12901,7 @@
       <c r="J278" t="n">
         <v>4130</v>
       </c>
-      <c r="K278"/>
+      <c r="K278" s="1"/>
       <c r="L278" t="n">
         <v>2022</v>
       </c>
@@ -12940,7 +12946,7 @@
       <c r="J279" t="n">
         <v>4130</v>
       </c>
-      <c r="K279"/>
+      <c r="K279" s="1"/>
       <c r="L279" t="n">
         <v>2022</v>
       </c>
@@ -12985,7 +12991,7 @@
       <c r="J280" t="n">
         <v>4130</v>
       </c>
-      <c r="K280"/>
+      <c r="K280" s="1"/>
       <c r="L280" t="n">
         <v>2022</v>
       </c>
@@ -13030,7 +13036,7 @@
       <c r="J281" t="n">
         <v>4130</v>
       </c>
-      <c r="K281"/>
+      <c r="K281" s="1"/>
       <c r="L281" t="n">
         <v>2022</v>
       </c>
@@ -13075,7 +13081,7 @@
       <c r="J282" t="n">
         <v>4130</v>
       </c>
-      <c r="K282"/>
+      <c r="K282" s="1"/>
       <c r="L282" t="n">
         <v>2022</v>
       </c>
@@ -13120,7 +13126,7 @@
       <c r="J283" t="n">
         <v>4130</v>
       </c>
-      <c r="K283"/>
+      <c r="K283" s="1"/>
       <c r="L283" t="n">
         <v>2022</v>
       </c>
@@ -13165,7 +13171,7 @@
       <c r="J284" t="n">
         <v>4130</v>
       </c>
-      <c r="K284"/>
+      <c r="K284" s="1"/>
       <c r="L284" t="n">
         <v>2022</v>
       </c>
@@ -13210,7 +13216,7 @@
       <c r="J285" t="n">
         <v>4130</v>
       </c>
-      <c r="K285"/>
+      <c r="K285" s="1"/>
       <c r="L285" t="n">
         <v>2023</v>
       </c>
@@ -13255,7 +13261,7 @@
       <c r="J286" t="n">
         <v>4130</v>
       </c>
-      <c r="K286"/>
+      <c r="K286" s="1"/>
       <c r="L286" t="n">
         <v>2023</v>
       </c>
@@ -13300,7 +13306,7 @@
       <c r="J287" t="n">
         <v>4130</v>
       </c>
-      <c r="K287"/>
+      <c r="K287" s="1"/>
       <c r="L287" t="n">
         <v>2024</v>
       </c>
@@ -13345,7 +13351,7 @@
       <c r="J288" t="n">
         <v>4130</v>
       </c>
-      <c r="K288"/>
+      <c r="K288" s="1"/>
       <c r="L288" t="n">
         <v>2024</v>
       </c>

</xml_diff>